<commit_message>
Corrige rangos de las formulas de resumen y el conteo de estados
Las cuatro formulas de la hoja Instrucciones que apuntan a la hoja de
ponentes arrancaban en la fila del encabezado (fila 3) en lugar de la
primera fila de datos (fila 4), de modo que contaban el titulo de columna
y omitian al ultimo docente. Rangos corregidos a las filas 4 a 18.

Ajusta ademas el desglose del mensaje de coordinacion: son 10 clases con
ponente por confirmar y 1 con el nombre incompleto, no 11 en un solo
grupo (8 + 10 + 1 + 9 = 28).

LibreOffice no se ejecuta en este entorno, por lo que las formulas se
verificaron reproduciendo COUNTA, COUNTIF y SUM sobre las celdas reales
del libro.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019GZ8Kkm9KwxHQZEVf8yg4N
</commit_message>
<xml_diff>
--- a/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
+++ b/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
@@ -708,7 +708,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:D28"/>
+  <dimension ref="A1:D28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -717,6 +717,7 @@
     <col width="16" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -745,6 +746,7 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
     <row r="7">
       <c r="B7" s="5" t="inlineStr">
         <is>
@@ -790,6 +792,7 @@
         </is>
       </c>
     </row>
+    <row r="11"/>
     <row r="12">
       <c r="B12" s="5" t="inlineStr">
         <is>
@@ -847,6 +850,7 @@
         </is>
       </c>
     </row>
+    <row r="17"/>
     <row r="18">
       <c r="B18" s="5" t="inlineStr">
         <is>
@@ -916,7 +920,7 @@
       </c>
       <c r="C23" s="16" t="n"/>
       <c r="D23" s="17">
-        <f>COUNTA('Ponentes - datos aval'!B3:B17)</f>
+        <f>COUNTA('Ponentes - datos aval'!B4:B18)</f>
         <v/>
       </c>
     </row>
@@ -928,7 +932,7 @@
       </c>
       <c r="C24" s="16" t="n"/>
       <c r="D24" s="17">
-        <f>COUNTIF('Ponentes - datos aval'!J3:J17,"SÍ")</f>
+        <f>COUNTIF('Ponentes - datos aval'!J4:J18,"SÍ")</f>
         <v/>
       </c>
     </row>
@@ -940,7 +944,7 @@
       </c>
       <c r="C25" s="16" t="n"/>
       <c r="D25" s="17">
-        <f>COUNTA('Ponentes - datos aval'!F3:F17)</f>
+        <f>COUNTA('Ponentes - datos aval'!F4:F18)</f>
         <v/>
       </c>
     </row>
@@ -952,10 +956,11 @@
       </c>
       <c r="C26" s="16" t="n"/>
       <c r="D26" s="17">
-        <f>COUNTIF('Ponentes - datos aval'!L3:L17,"SÍ")</f>
+        <f>COUNTIF('Ponentes - datos aval'!L4:L18,"SÍ")</f>
         <v/>
       </c>
     </row>
+    <row r="27"/>
     <row r="28" ht="40" customHeight="1">
       <c r="B28" s="18" t="inlineStr">
         <is>
@@ -2041,6 +2046,7 @@
         </is>
       </c>
     </row>
+    <row r="31"/>
     <row r="32">
       <c r="C32" s="31" t="inlineStr">
         <is>
@@ -2096,6 +2102,7 @@
         <v/>
       </c>
     </row>
+    <row r="37"/>
     <row r="38">
       <c r="C38" s="34" t="inlineStr">
         <is>
@@ -2132,7 +2139,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N21"/>
+  <dimension ref="A1:N24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2695,6 +2702,7 @@
         </is>
       </c>
     </row>
+    <row r="19"/>
     <row r="20">
       <c r="A20" s="46" t="inlineStr">
         <is>
@@ -2774,6 +2782,9 @@
         </is>
       </c>
     </row>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="J4:L18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">

</xml_diff>